<commit_message>
LSIM INTERP = FALSE
estimation_loop.py: when CURR_TIME_USER = -1, and the current date is after EoR, the last day will be selected automatically; at EoR, do not run optimize, use the estimate of current state as model prediction for EoR; ssm.py: changed lsim_mod's interp option to False to use the actual zeroth-order input instead of an interpolation of input so EoR u will not affect EoR pred; mpc_optimizer.py: added end_of_run option in optimize(); master data: fixed DO's unit on D12
</commit_message>
<xml_diff>
--- a/data/dmc-test-with-mr24-030-experiment-data/MR24-030-MasterDataTable.xlsx
+++ b/data/dmc-test-with-mr24-030-experiment-data/MR24-030-MasterDataTable.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://myteams.gsk.com/sites/BiopharmModelPredictiveControl/Shared Documents/General/data/MR24-030-MPC-3L/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yl604392\Git\state-space-model\data\dmc-test-with-mr24-030-experiment-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2166" documentId="8_{2425AED5-2B3D-4BFD-84B8-542313010F1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{62FE98CD-365A-49A1-A0B0-CB948C804BE8}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E8DED3A-3C1B-4640-9409-9FCAF12B5D2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3510" yWindow="3510" windowWidth="28800" windowHeight="15435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="MasterDataTable" sheetId="1" r:id="rId1"/>
@@ -1478,16 +1478,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BK70"/>
-  <sheetFormatPr defaultColWidth="14.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="4" width="10.6640625" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" customWidth="1"/>
-    <col min="6" max="60" width="12.6640625" customWidth="1"/>
-    <col min="61" max="61" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="62" max="63" width="16.33203125" customWidth="1"/>
+    <col min="2" max="4" width="10.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="6" max="60" width="12.7109375" customWidth="1"/>
+    <col min="61" max="61" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="62" max="63" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:63" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:63" ht="21" x14ac:dyDescent="0.35">
       <c r="A1" s="74" t="s">
         <v>0</v>
       </c>
@@ -1566,7 +1566,7 @@
       <c r="BJ1" s="79"/>
       <c r="BK1" s="80"/>
     </row>
-    <row r="2" spans="1:63" ht="60.6" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:63" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="33" t="s">
         <v>3</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="3" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>53</v>
       </c>
@@ -1953,7 +1953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>54</v>
       </c>
@@ -2151,7 +2151,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>55</v>
       </c>
@@ -2349,7 +2349,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>56</v>
       </c>
@@ -2545,7 +2545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>57</v>
       </c>
@@ -2746,7 +2746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>58</v>
       </c>
@@ -2947,7 +2947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
         <v>53</v>
       </c>
@@ -3146,7 +3146,7 @@
         <v>17.4800465</v>
       </c>
     </row>
-    <row r="10" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>54</v>
       </c>
@@ -3347,7 +3347,7 @@
         <v>17.745815000000004</v>
       </c>
     </row>
-    <row r="11" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>55</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>17.393346000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>56</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>21.373875000000002</v>
       </c>
     </row>
-    <row r="13" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>57</v>
       </c>
@@ -3950,7 +3950,7 @@
         <v>14.022246000000001</v>
       </c>
     </row>
-    <row r="14" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>58</v>
       </c>
@@ -4155,7 +4155,7 @@
         <v>17.715888</v>
       </c>
     </row>
-    <row r="15" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>53</v>
       </c>
@@ -4354,7 +4354,7 @@
         <v>11.539479000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>54</v>
       </c>
@@ -4555,7 +4555,7 @@
         <v>12.608789925000002</v>
       </c>
     </row>
-    <row r="17" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>55</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>11.993802225000001</v>
       </c>
     </row>
-    <row r="18" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>56</v>
       </c>
@@ -4945,7 +4945,7 @@
         <v>13.025639999999999</v>
       </c>
     </row>
-    <row r="19" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>57</v>
       </c>
@@ -5145,7 +5145,7 @@
         <v>3.9633683594627347</v>
       </c>
     </row>
-    <row r="20" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>58</v>
       </c>
@@ -5348,7 +5348,7 @@
         <v>8.4828514616618094</v>
       </c>
     </row>
-    <row r="21" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
         <v>53</v>
       </c>
@@ -5547,7 +5547,7 @@
         <v>13.18215</v>
       </c>
     </row>
-    <row r="22" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>54</v>
       </c>
@@ -5748,7 +5748,7 @@
         <v>13.150274999999999</v>
       </c>
     </row>
-    <row r="23" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>55</v>
       </c>
@@ -5949,7 +5949,7 @@
         <v>13.12635</v>
       </c>
     </row>
-    <row r="24" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>57</v>
       </c>
@@ -6152,7 +6152,7 @@
         <v>5.3590759753051112</v>
       </c>
     </row>
-    <row r="25" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="6" t="s">
         <v>58</v>
       </c>
@@ -6355,7 +6355,7 @@
         <v>7.4775654747660001</v>
       </c>
     </row>
-    <row r="26" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>53</v>
       </c>
@@ -6554,7 +6554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>54</v>
       </c>
@@ -6755,7 +6755,7 @@
         <v>6.7380460000000006</v>
       </c>
     </row>
-    <row r="28" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>55</v>
       </c>
@@ -6956,7 +6956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>57</v>
       </c>
@@ -7156,7 +7156,7 @@
         <v>4.2185063447336155</v>
       </c>
     </row>
-    <row r="30" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>58</v>
       </c>
@@ -7356,7 +7356,7 @@
         <v>3.6766410485124208</v>
       </c>
     </row>
-    <row r="31" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A31" s="3" t="s">
         <v>53</v>
       </c>
@@ -7555,7 +7555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>54</v>
       </c>
@@ -7756,7 +7756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>55</v>
       </c>
@@ -7957,7 +7957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>57</v>
       </c>
@@ -8160,7 +8160,7 @@
         <v>7.6791147043425241</v>
       </c>
     </row>
-    <row r="35" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="6" t="s">
         <v>58</v>
       </c>
@@ -8363,7 +8363,7 @@
         <v>10.261394893996174</v>
       </c>
     </row>
-    <row r="36" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>53</v>
       </c>
@@ -8560,7 +8560,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>54</v>
       </c>
@@ -8759,7 +8759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>55</v>
       </c>
@@ -8958,7 +8958,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>57</v>
       </c>
@@ -9156,7 +9156,7 @@
         <v>8.4915585188980369</v>
       </c>
     </row>
-    <row r="40" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>58</v>
       </c>
@@ -9357,7 +9357,7 @@
         <v>2.3220682771976411</v>
       </c>
     </row>
-    <row r="41" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A41" s="3" t="s">
         <v>53</v>
       </c>
@@ -9554,7 +9554,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>54</v>
       </c>
@@ -9753,7 +9753,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>55</v>
       </c>
@@ -9952,7 +9952,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>57</v>
       </c>
@@ -10153,7 +10153,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
         <v>58</v>
       </c>
@@ -10354,7 +10354,7 @@
         <v>3.0977345708595014</v>
       </c>
     </row>
-    <row r="46" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>53</v>
       </c>
@@ -10549,7 +10549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>54</v>
       </c>
@@ -10746,7 +10746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>55</v>
       </c>
@@ -10943,7 +10943,7 @@
         <v>9.5097380000000022</v>
       </c>
     </row>
-    <row r="49" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>57</v>
       </c>
@@ -11142,7 +11142,7 @@
         <v>6.6672711206767126</v>
       </c>
     </row>
-    <row r="50" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>58</v>
       </c>
@@ -11341,7 +11341,7 @@
         <v>6.8219871831206671</v>
       </c>
     </row>
-    <row r="51" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A51" s="3" t="s">
         <v>53</v>
       </c>
@@ -11538,7 +11538,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>54</v>
       </c>
@@ -11737,7 +11737,7 @@
         <v>14.179864050000001</v>
       </c>
     </row>
-    <row r="53" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>55</v>
       </c>
@@ -11936,7 +11936,7 @@
         <v>9.8582900000000002</v>
       </c>
     </row>
-    <row r="54" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>57</v>
       </c>
@@ -12137,7 +12137,7 @@
         <v>1.2053112985361027</v>
       </c>
     </row>
-    <row r="55" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A55" s="6" t="s">
         <v>58</v>
       </c>
@@ -12338,7 +12338,7 @@
         <v>5.7991313075208026</v>
       </c>
     </row>
-    <row r="56" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>53</v>
       </c>
@@ -12535,7 +12535,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>54</v>
       </c>
@@ -12734,7 +12734,7 @@
         <v>12.103236375000002</v>
       </c>
     </row>
-    <row r="58" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>55</v>
       </c>
@@ -12933,7 +12933,7 @@
         <v>10.504482600000001</v>
       </c>
     </row>
-    <row r="59" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -13134,7 +13134,7 @@
         <v>6.9891921680878912</v>
       </c>
     </row>
-    <row r="60" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -13335,7 +13335,7 @@
         <v>7.1864023795214536</v>
       </c>
     </row>
-    <row r="61" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A61" s="3" t="s">
         <v>53</v>
       </c>
@@ -13532,7 +13532,7 @@
         <v>9.7536480000000001</v>
       </c>
     </row>
-    <row r="62" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>54</v>
       </c>
@@ -13731,7 +13731,7 @@
         <v>11.520405</v>
       </c>
     </row>
-    <row r="63" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>55</v>
       </c>
@@ -13930,7 +13930,7 @@
         <v>14.508377000000003</v>
       </c>
     </row>
-    <row r="64" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>57</v>
       </c>
@@ -14129,7 +14129,7 @@
         <v>5.8497357969925208</v>
       </c>
     </row>
-    <row r="65" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
         <v>58</v>
       </c>
@@ -14330,7 +14330,7 @@
         <v>1.9961199999999997E-4</v>
       </c>
     </row>
-    <row r="66" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A66" s="3" t="s">
         <v>53</v>
       </c>
@@ -14417,7 +14417,7 @@
         <v>299</v>
       </c>
       <c r="AD66" s="4">
-        <v>50.1</v>
+        <v>0.501</v>
       </c>
       <c r="AE66" s="4">
         <v>7.3</v>
@@ -14524,7 +14524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>54</v>
       </c>
@@ -14611,7 +14611,7 @@
         <v>300</v>
       </c>
       <c r="AD67" s="27">
-        <v>50.8</v>
+        <v>0.50800000000000001</v>
       </c>
       <c r="AE67" s="27">
         <v>7.12</v>
@@ -14718,7 +14718,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>55</v>
       </c>
@@ -14805,7 +14805,7 @@
         <v>302</v>
       </c>
       <c r="AD68" s="27">
-        <v>49.1</v>
+        <v>0.49099999999999999</v>
       </c>
       <c r="AE68" s="27">
         <v>7.3</v>
@@ -14912,7 +14912,7 @@
         <v>12.26869175</v>
       </c>
     </row>
-    <row r="69" spans="1:63" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:63" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>57</v>
       </c>
@@ -14999,7 +14999,7 @@
         <v>301</v>
       </c>
       <c r="AD69" s="27">
-        <v>49.7</v>
+        <v>0.49700000000000005</v>
       </c>
       <c r="AE69" s="27">
         <v>7.3</v>
@@ -15106,7 +15106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:63" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:63" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A70" s="6" t="s">
         <v>58</v>
       </c>
@@ -15193,7 +15193,7 @@
         <v>302</v>
       </c>
       <c r="AD70" s="7">
-        <v>50.3</v>
+        <v>0.503</v>
       </c>
       <c r="AE70" s="7">
         <v>7.3</v>
@@ -15335,13 +15335,40 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A841E7D6-1405-4AC8-A599-0CE4601ECD66}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B75172DAFC2BB6479729CB287362C7E3" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0fc11b0946794a47057850b4f6c92dd7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="34d8c884-fe7e-4d4f-a833-b92a2823f74b" xmlns:ns3="a198008e-c7f6-4ed0-9865-26ace3c97b59" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fb90ec7fe59ed1d44226abab88cd233b" ns2:_="" ns3:_="">
     <xsd:import namespace="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
@@ -15564,34 +15591,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
+    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="34d8c884-fe7e-4d4f-a833-b92a2823f74b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="a198008e-c7f6-4ed0-9865-26ace3c97b59">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9F43DC28-AE43-4EFF-8739-4E0C557B415B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -15608,29 +15633,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6FA2C79D-5C43-4F8C-8CB2-6CBFC4591548}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{81736866-79EE-4C47-B374-7C3565856A36}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="a198008e-c7f6-4ed0-9865-26ace3c97b59"/>
-    <ds:schemaRef ds:uri="34d8c884-fe7e-4d4f-a833-b92a2823f74b"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>